<commit_message>
Preenchendo tabela de validacao e registrando resultados em planilha
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Registro de treinamento - Adaline.xlsx
+++ b/Registro de treinamento - Adaline.xlsx
@@ -638,39 +638,39 @@
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.8194389077364684</v>
+        <v>0.712955486664269</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.2067497825636504</v>
+        <v>0.02264741942114035</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>0.6227125553188931</v>
+        <v>0.2072144159849879</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>0.02506774222266372</v>
+        <v>0.735784669848443</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>0.7404231242345561</v>
+        <v>0.1484238348529446</v>
       </c>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="10" t="n">
-        <v>-1.463959786774032</v>
+        <v>-1.46395166500966</v>
       </c>
       <c r="M8" s="10" t="n">
-        <v>1.445345167074975</v>
+        <v>1.445424092681469</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>1.391009641054352</v>
+        <v>1.391106343053838</v>
       </c>
       <c r="O8" s="10" t="n">
-        <v>-0.4754358955153574</v>
+        <v>-0.4752706983151977</v>
       </c>
       <c r="P8" s="10" t="n">
-        <v>-1.052115960746899</v>
+        <v>-1.052171315787007</v>
       </c>
       <c r="Q8" s="6" t="n"/>
       <c r="R8" s="1" t="n">
-        <v>873</v>
+        <v>895</v>
       </c>
     </row>
     <row r="9">
@@ -680,39 +680,39 @@
         </is>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.9564542749895671</v>
+        <v>0.1916743680109427</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>0.776203222955592</v>
+        <v>0.7158984841011907</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0.3183518919651893</v>
+        <v>0.9297230448023421</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>0.1053166479606685</v>
+        <v>0.5692327204078355</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.3268968153278473</v>
+        <v>0.8471791855487361</v>
       </c>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="10" t="n">
-        <v>-1.463959014276096</v>
+        <v>-1.463895979247844</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>1.445386371388172</v>
+        <v>1.445428080280017</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>1.391061118436364</v>
+        <v>1.391094691483407</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>-0.475353356388255</v>
+        <v>-0.4752049894941972</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-1.052145673157537</v>
+        <v>-1.052160746939282</v>
       </c>
       <c r="Q9" s="6" t="n"/>
       <c r="R9" s="1" t="n">
-        <v>879</v>
+        <v>847</v>
       </c>
     </row>
     <row r="10">
@@ -722,39 +722,39 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.424692428669886</v>
+        <v>0.5500845014098341</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.3205935555667212</v>
+        <v>0.8398379697443172</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>0.4062393887508391</v>
+        <v>0.6635540082324423</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>0.3269943806882403</v>
+        <v>0.8103578145537644</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.1604169390486379</v>
+        <v>0.004045743261202439</v>
       </c>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="10" t="n">
-        <v>-1.464002043615717</v>
+        <v>-1.463883678119296</v>
       </c>
       <c r="M10" s="10" t="n">
-        <v>1.445381312095036</v>
+        <v>1.445487416851732</v>
       </c>
       <c r="N10" s="10" t="n">
-        <v>1.391067701853915</v>
+        <v>1.391165504113729</v>
       </c>
       <c r="O10" s="10" t="n">
-        <v>-0.4754079070005145</v>
+        <v>-0.4750744470114993</v>
       </c>
       <c r="P10" s="10" t="n">
-        <v>-1.052152439339208</v>
+        <v>-1.052200845649805</v>
       </c>
       <c r="Q10" s="6" t="n"/>
       <c r="R10" s="1" t="n">
-        <v>856</v>
+        <v>867</v>
       </c>
     </row>
     <row r="11">
@@ -764,39 +764,39 @@
         </is>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.06460488382519169</v>
+        <v>0.7557309744702216</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>0.4523580328372858</v>
+        <v>0.2048433627592801</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>0.2712387667855974</v>
+        <v>0.01654229849491273</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>0.4236803027551156</v>
+        <v>0.3935456051946653</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>0.6109391376627016</v>
+        <v>0.04901086926316811</v>
       </c>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="10" t="n">
-        <v>-1.463970645113263</v>
+        <v>-1.46386753401028</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>1.445358510836584</v>
+        <v>1.44536972713341</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>1.391029681042357</v>
+        <v>1.391012886411653</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>-0.4754205849682122</v>
+        <v>-0.4752913817108214</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>-1.052128294574105</v>
+        <v>-1.052111489250867</v>
       </c>
       <c r="Q11" s="6" t="n"/>
       <c r="R11" s="1" t="n">
-        <v>851</v>
+        <v>886</v>
       </c>
     </row>
     <row r="12">
@@ -806,39 +806,39 @@
         </is>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.09066872789956837</v>
+        <v>0.9576976872948032</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.9962416819217922</v>
+        <v>0.04742169366131121</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>0.1471707682439249</v>
+        <v>0.4941165635831412</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>0.1400186055989903</v>
+        <v>0.3397032219787661</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>0.6199105902321989</v>
+        <v>0.243702033529164</v>
       </c>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="10" t="n">
-        <v>-1.4639823178641</v>
+        <v>-1.463886930081521</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>1.445328955233634</v>
+        <v>1.445384635813414</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>1.390995986506527</v>
+        <v>1.3910374158738</v>
       </c>
       <c r="O12" s="10" t="n">
-        <v>-0.4754915569215959</v>
+        <v>-0.4752818948697449</v>
       </c>
       <c r="P12" s="10" t="n">
-        <v>-1.052109616639759</v>
+        <v>-1.052127007041477</v>
       </c>
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="1" t="n">
-        <v>839</v>
+        <v>887</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajuste na logica do treinamento
</commit_message>
<xml_diff>
--- a/Registro de treinamento - Adaline.xlsx
+++ b/Registro de treinamento - Adaline.xlsx
@@ -638,39 +638,39 @@
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.712955486664269</v>
+        <v>0.00749930518219355</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.02264741942114035</v>
+        <v>0.6942400655620203</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>0.2072144159849879</v>
+        <v>0.9569092545181411</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>0.735784669848443</v>
+        <v>0.06487294772074248</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>0.1484238348529446</v>
+        <v>0.003374603364497131</v>
       </c>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="10" t="n">
-        <v>-1.46395166500966</v>
+        <v>-1.463934704095472</v>
       </c>
       <c r="M8" s="10" t="n">
-        <v>1.445424092681469</v>
+        <v>1.44534284101754</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>1.391106343053838</v>
+        <v>1.390999288845007</v>
       </c>
       <c r="O8" s="10" t="n">
-        <v>-0.4752706983151977</v>
+        <v>-0.4754143117748792</v>
       </c>
       <c r="P8" s="10" t="n">
-        <v>-1.052171315787007</v>
+        <v>-1.052108247541798</v>
       </c>
       <c r="Q8" s="6" t="n"/>
       <c r="R8" s="1" t="n">
-        <v>895</v>
+        <v>786</v>
       </c>
     </row>
     <row r="9">
@@ -680,39 +680,39 @@
         </is>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.1916743680109427</v>
+        <v>0.04706589351040469</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>0.7158984841011907</v>
+        <v>0.2799283539729676</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0.9297230448023421</v>
+        <v>0.6478158707917085</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>0.5692327204078355</v>
+        <v>0.1482316449724698</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.8471791855487361</v>
+        <v>0.6478864329706511</v>
       </c>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="10" t="n">
-        <v>-1.463895979247844</v>
+        <v>-1.464043241143429</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>1.445428080280017</v>
+        <v>1.445315605885658</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>1.391094691483407</v>
+        <v>1.390997564277824</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>-0.4752049894941972</v>
+        <v>-0.4755810173510531</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-1.052160746939282</v>
+        <v>-1.052114718735778</v>
       </c>
       <c r="Q9" s="6" t="n"/>
       <c r="R9" s="1" t="n">
-        <v>847</v>
+        <v>828</v>
       </c>
     </row>
     <row r="10">
@@ -722,39 +722,39 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.5500845014098341</v>
+        <v>0.926355874084188</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.8398379697443172</v>
+        <v>0.6791061100312741</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>0.6635540082324423</v>
+        <v>0.5751946399107339</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>0.8103578145537644</v>
+        <v>0.9233144178610824</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.004045743261202439</v>
+        <v>0.09462061029006918</v>
       </c>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="10" t="n">
-        <v>-1.463883678119296</v>
+        <v>-1.463954867406505</v>
       </c>
       <c r="M10" s="10" t="n">
-        <v>1.445487416851732</v>
+        <v>1.445495251385341</v>
       </c>
       <c r="N10" s="10" t="n">
-        <v>1.391165504113729</v>
+        <v>1.391196637123609</v>
       </c>
       <c r="O10" s="10" t="n">
-        <v>-0.4750744470114993</v>
+        <v>-0.4751327760903527</v>
       </c>
       <c r="P10" s="10" t="n">
-        <v>-1.052200845649805</v>
+        <v>-1.052223745763968</v>
       </c>
       <c r="Q10" s="6" t="n"/>
       <c r="R10" s="1" t="n">
-        <v>867</v>
+        <v>897</v>
       </c>
     </row>
     <row r="11">
@@ -764,39 +764,39 @@
         </is>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.7557309744702216</v>
+        <v>0.5012086227767798</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>0.2048433627592801</v>
+        <v>0.6850885482940736</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>0.01654229849491273</v>
+        <v>0.2187994576835838</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>0.3935456051946653</v>
+        <v>0.2655385418448383</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>0.04901086926316811</v>
+        <v>0.8693193060990763</v>
       </c>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="10" t="n">
-        <v>-1.46386753401028</v>
+        <v>-1.464020180207643</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>1.44536972713341</v>
+        <v>1.445376406570885</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>1.391012886411653</v>
+        <v>1.391066923665506</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>-0.4752913817108214</v>
+        <v>-0.4754365736510865</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>-1.052111489250867</v>
+        <v>-1.052153238259929</v>
       </c>
       <c r="Q11" s="6" t="n"/>
       <c r="R11" s="1" t="n">
-        <v>886</v>
+        <v>875</v>
       </c>
     </row>
     <row r="12">
@@ -806,39 +806,39 @@
         </is>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.9576976872948032</v>
+        <v>0.3047356559891302</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.04742169366131121</v>
+        <v>0.3949626530683568</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>0.4941165635831412</v>
+        <v>0.8567140245921021</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>0.3397032219787661</v>
+        <v>0.7861557189827201</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>0.243702033529164</v>
+        <v>0.5099104312468491</v>
       </c>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="10" t="n">
-        <v>-1.463886930081521</v>
+        <v>-1.463920717504418</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>1.445384635813414</v>
+        <v>1.44545608016262</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>1.3910374158738</v>
+        <v>1.391137277481289</v>
       </c>
       <c r="O12" s="10" t="n">
-        <v>-0.4752818948697449</v>
+        <v>-0.4751750070000684</v>
       </c>
       <c r="P12" s="10" t="n">
-        <v>-1.052127007041477</v>
+        <v>-1.05218707245827</v>
       </c>
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="1" t="n">
-        <v>887</v>
+        <v>861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Plotando o grafico do erro quadratico medio (EQM) em função da época para cada treinamento e salvando as imagens na pasta Graphics.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Registro de treinamento - Adaline.xlsx
+++ b/Registro de treinamento - Adaline.xlsx
@@ -638,39 +638,39 @@
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.00749930518219355</v>
+        <v>0.4442387535505021</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.6942400655620203</v>
+        <v>0.7800443928443846</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>0.9569092545181411</v>
+        <v>0.353275187596967</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>0.06487294772074248</v>
+        <v>0.2175351937567953</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>0.003374603364497131</v>
+        <v>0.8189864002005304</v>
       </c>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="10" t="n">
-        <v>-1.463934704095472</v>
+        <v>-1.46398381586319</v>
       </c>
       <c r="M8" s="10" t="n">
-        <v>1.44534284101754</v>
+        <v>1.445368776061362</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>1.390999288845007</v>
+        <v>1.391046456243668</v>
       </c>
       <c r="O8" s="10" t="n">
-        <v>-0.4754143117748792</v>
+        <v>-0.4754140018734558</v>
       </c>
       <c r="P8" s="10" t="n">
-        <v>-1.052108247541798</v>
+        <v>-1.052138901624593</v>
       </c>
       <c r="Q8" s="6" t="n"/>
       <c r="R8" s="1" t="n">
-        <v>786</v>
+        <v>864</v>
       </c>
     </row>
     <row r="9">
@@ -680,39 +680,39 @@
         </is>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.04706589351040469</v>
+        <v>0.7766602728401847</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>0.2799283539729676</v>
+        <v>0.9939852324239665</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0.6478158707917085</v>
+        <v>0.547302585126985</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>0.1482316449724698</v>
+        <v>0.6835108293955193</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.6478864329706511</v>
+        <v>0.9492817554032504</v>
       </c>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="10" t="n">
-        <v>-1.464043241143429</v>
+        <v>-1.463976774954467</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>1.445315605885658</v>
+        <v>1.445461259429519</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>1.390997564277824</v>
+        <v>1.391160487047401</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>-0.4755810173510531</v>
+        <v>-0.4752230520085841</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-1.052114718735778</v>
+        <v>-1.052204351175279</v>
       </c>
       <c r="Q9" s="6" t="n"/>
       <c r="R9" s="1" t="n">
-        <v>828</v>
+        <v>895</v>
       </c>
     </row>
     <row r="10">
@@ -722,39 +722,39 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.926355874084188</v>
+        <v>0.4276366157881288</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.6791061100312741</v>
+        <v>0.9419000297673071</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>0.5751946399107339</v>
+        <v>0.208553745416867</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>0.9233144178610824</v>
+        <v>0.2287246302928339</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.09462061029006918</v>
+        <v>0.02463832146568345</v>
       </c>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="10" t="n">
-        <v>-1.463954867406505</v>
+        <v>-1.463960295849152</v>
       </c>
       <c r="M10" s="10" t="n">
-        <v>1.445495251385341</v>
+        <v>1.445384000961064</v>
       </c>
       <c r="N10" s="10" t="n">
-        <v>1.391196637123609</v>
+        <v>1.39105852619042</v>
       </c>
       <c r="O10" s="10" t="n">
-        <v>-0.4751327760903527</v>
+        <v>-0.4753593908387779</v>
       </c>
       <c r="P10" s="10" t="n">
-        <v>-1.052223745763968</v>
+        <v>-1.052144262452725</v>
       </c>
       <c r="Q10" s="6" t="n"/>
       <c r="R10" s="1" t="n">
-        <v>897</v>
+        <v>849</v>
       </c>
     </row>
     <row r="11">
@@ -764,39 +764,39 @@
         </is>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.5012086227767798</v>
+        <v>0.6475155468846241</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>0.6850885482940736</v>
+        <v>0.08986157157178287</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>0.2187994576835838</v>
+        <v>0.08645484215915178</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>0.2655385418448383</v>
+        <v>0.18492123928513</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>0.8693193060990763</v>
+        <v>0.3617567741826059</v>
       </c>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="10" t="n">
-        <v>-1.464020180207643</v>
+        <v>-1.463947960301699</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>1.445376406570885</v>
+        <v>1.445338510350447</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>1.391066923665506</v>
+        <v>1.390997754391377</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>-0.4754365736510865</v>
+        <v>-0.4754368149829555</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>-1.052153238259929</v>
+        <v>-1.05210827372784</v>
       </c>
       <c r="Q11" s="6" t="n"/>
       <c r="R11" s="1" t="n">
-        <v>875</v>
+        <v>878</v>
       </c>
     </row>
     <row r="12">
@@ -806,39 +806,39 @@
         </is>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.3047356559891302</v>
+        <v>0.02180824250306634</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.3949626530683568</v>
+        <v>0.972761972170046</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>0.8567140245921021</v>
+        <v>0.2071343968798602</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>0.7861557189827201</v>
+        <v>0.9276847012545675</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>0.5099104312468491</v>
+        <v>0.5200279362472735</v>
       </c>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="10" t="n">
-        <v>-1.463920717504418</v>
+        <v>-1.464000137960732</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>1.44545608016262</v>
+        <v>1.445470797414762</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>1.391137277481289</v>
+        <v>1.391179483540758</v>
       </c>
       <c r="O12" s="10" t="n">
-        <v>-0.4751750070000684</v>
+        <v>-0.4752282883345668</v>
       </c>
       <c r="P12" s="10" t="n">
-        <v>-1.05218707245827</v>
+        <v>-1.052216942199985</v>
       </c>
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="1" t="n">
-        <v>861</v>
+        <v>865</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalização do projeto Adaline: adição de métricas de classificação, gráficos de matriz de confusão e relatório em txt.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Registro de treinamento - Adaline.xlsx
+++ b/Registro de treinamento - Adaline.xlsx
@@ -638,39 +638,39 @@
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.4442387535505021</v>
+        <v>0.583509973089374</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.7800443928443846</v>
+        <v>0.9134266270806541</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>0.353275187596967</v>
+        <v>0.3544153112726233</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>0.2175351937567953</v>
+        <v>0.5816550928565771</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>0.8189864002005304</v>
+        <v>0.556188398851772</v>
       </c>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="10" t="n">
-        <v>-1.46398381586319</v>
+        <v>-1.463882314170113</v>
       </c>
       <c r="M8" s="10" t="n">
-        <v>1.445368776061362</v>
+        <v>1.445425209877661</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>1.391046456243668</v>
+        <v>1.39108695766525</v>
       </c>
       <c r="O8" s="10" t="n">
-        <v>-0.4754140018734558</v>
+        <v>-0.4751966051348737</v>
       </c>
       <c r="P8" s="10" t="n">
-        <v>-1.052138901624593</v>
+        <v>-1.05215533568717</v>
       </c>
       <c r="Q8" s="6" t="n"/>
       <c r="R8" s="1" t="n">
-        <v>864</v>
+        <v>879</v>
       </c>
     </row>
     <row r="9">
@@ -680,39 +680,39 @@
         </is>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.7766602728401847</v>
+        <v>0.4571674324798281</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>0.9939852324239665</v>
+        <v>0.1302496392054713</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0.547302585126985</v>
+        <v>0.08930069358077097</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>0.6835108293955193</v>
+        <v>0.06789109164875406</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.9492817554032504</v>
+        <v>0.6324117007931139</v>
       </c>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="10" t="n">
-        <v>-1.463976774954467</v>
+        <v>-1.463960778611721</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>1.445461259429519</v>
+        <v>1.445302802254618</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>1.391160487047401</v>
+        <v>1.390956751800876</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>-0.4752230520085841</v>
+        <v>-0.4755210144201079</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-1.052204351175279</v>
+        <v>-1.052085447477972</v>
       </c>
       <c r="Q9" s="6" t="n"/>
       <c r="R9" s="1" t="n">
-        <v>895</v>
+        <v>868</v>
       </c>
     </row>
     <row r="10">
@@ -722,39 +722,39 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.4276366157881288</v>
+        <v>0.8812485387199801</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.9419000297673071</v>
+        <v>0.3734062729525122</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>0.208553745416867</v>
+        <v>0.3214906019414109</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>0.2287246302928339</v>
+        <v>0.4708680220256262</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.02463832146568345</v>
+        <v>0.7384733125368648</v>
       </c>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="10" t="n">
-        <v>-1.463960295849152</v>
+        <v>-1.463926308329083</v>
       </c>
       <c r="M10" s="10" t="n">
-        <v>1.445384000961064</v>
+        <v>1.445402557609132</v>
       </c>
       <c r="N10" s="10" t="n">
-        <v>1.39105852619042</v>
+        <v>1.391071687398528</v>
       </c>
       <c r="O10" s="10" t="n">
-        <v>-0.4753593908387779</v>
+        <v>-0.4752872088395602</v>
       </c>
       <c r="P10" s="10" t="n">
-        <v>-1.052144262452725</v>
+        <v>-1.052149533196757</v>
       </c>
       <c r="Q10" s="6" t="n"/>
       <c r="R10" s="1" t="n">
-        <v>849</v>
+        <v>899</v>
       </c>
     </row>
     <row r="11">
@@ -764,39 +764,39 @@
         </is>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.6475155468846241</v>
+        <v>0.10358911268268</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>0.08986157157178287</v>
+        <v>0.501129039561431</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>0.08645484215915178</v>
+        <v>0.7163161191544168</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>0.18492123928513</v>
+        <v>0.7913196967331946</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>0.3617567741826059</v>
+        <v>0.3708843418107386</v>
       </c>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="10" t="n">
-        <v>-1.463947960301699</v>
+        <v>-1.463849134320305</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>1.445338510350447</v>
+        <v>1.44544205802979</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>1.390997754391377</v>
+        <v>1.391098263727202</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>-0.4754368149829555</v>
+        <v>-0.4751285385881502</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>-1.05210827372784</v>
+        <v>-1.052159588347229</v>
       </c>
       <c r="Q11" s="6" t="n"/>
       <c r="R11" s="1" t="n">
-        <v>878</v>
+        <v>849</v>
       </c>
     </row>
     <row r="12">
@@ -806,39 +806,39 @@
         </is>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.02180824250306634</v>
+        <v>0.7661249439788895</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.972761972170046</v>
+        <v>0.4454533001567049</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>0.2071343968798602</v>
+        <v>0.5400723749640246</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>0.9276847012545675</v>
+        <v>0.5235431112000402</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>0.5200279362472735</v>
+        <v>0.3873266145845546</v>
       </c>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="10" t="n">
-        <v>-1.464000137960732</v>
+        <v>-1.463868132853051</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>1.445470797414762</v>
+        <v>1.445413508808737</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>1.391179483540758</v>
+        <v>1.391068041411476</v>
       </c>
       <c r="O12" s="10" t="n">
-        <v>-0.4752282883345668</v>
+        <v>-0.4752050749940616</v>
       </c>
       <c r="P12" s="10" t="n">
-        <v>-1.052216942199985</v>
+        <v>-1.05214342184153</v>
       </c>
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="1" t="n">
-        <v>865</v>
+        <v>882</v>
       </c>
     </row>
   </sheetData>

</xml_diff>